<commit_message>
Corrige perda de valores decimais em Orcamento, Valor e Diaria
- Campos numericos (Orcamento da obra, Valor da movimentacao, Diaria do dia trabalhado) usavam input type=number, que rejeita silenciosamente virgula como separador decimal (formato BR), zerando o valor ao salvar
- Troca para input de texto com parseValorBR(), aceitando tanto "75.000,50" (BR) quanto "75000.50"
- Adiciona numToInputBR() para exibir o valor ja formatado com virgula ao reabrir um registro para edicao
- Corrige chave "Status" duplicada nos objetos de Obras e Movimentacoes na exportacao para Excel, que sobrescrevia o status de auditoria (C/A/D); renomeada para "Status Auditoria"
- Atualiza GestaoMultiServicos.xlsx com os lancamentos registrados durante o uso local

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/GestaoMultiServicos.xlsx
+++ b/GestaoMultiServicos.xlsx
@@ -403,11 +403,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status</v>
+        <v>Status Auditoria</v>
       </c>
       <c r="B1" t="str">
         <v>Data/Hora</v>
@@ -449,24 +449,27 @@
         <v>Vencimento</v>
       </c>
       <c r="O1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="P1" t="str">
         <v>Data Pag.</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Gerador</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Recebido</v>
+        <v>D</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>26/06/2026 11:53:32</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D2" t="str">
-        <v>v2y7nnmu</v>
+        <v>8y5c5ibr</v>
       </c>
       <c r="E2" t="str">
         <v>Recebimento</v>
@@ -481,7 +484,7 @@
         <v>DPBEA</v>
       </c>
       <c r="I2" t="str">
-        <v>NF 1234</v>
+        <v>Inicio das obras</v>
       </c>
       <c r="J2">
         <v>10000</v>
@@ -496,27 +499,30 @@
         <v/>
       </c>
       <c r="N2" t="str">
-        <v>2026-06-24</v>
+        <v>2026-06-10</v>
       </c>
       <c r="O2" t="str">
-        <v>2026-06-20</v>
+        <v>Recebido</v>
       </c>
       <c r="P2" t="str">
+        <v>2026-06-10</v>
+      </c>
+      <c r="Q2" t="str">
         <v>Sim</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Pago</v>
+        <v>D</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>26/06/2026 11:53:34</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D3" t="str">
-        <v>dnspp1sf</v>
+        <v>9wjucmk0</v>
       </c>
       <c r="E3" t="str">
         <v>Despesa</v>
@@ -528,16 +534,16 @@
         <v>Sergio Tarnta</v>
       </c>
       <c r="H3" t="str">
-        <v>DPBEA</v>
+        <v>Armazem - Cajamar</v>
       </c>
       <c r="I3" t="str">
-        <v>Diária: Sergio Tarnta — DPBEA (Demolição)</v>
+        <v>Instalação de painel</v>
       </c>
       <c r="J3">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="K3" t="str">
-        <v>PIX</v>
+        <v>À vista</v>
       </c>
       <c r="L3" t="str">
         <v/>
@@ -546,27 +552,30 @@
         <v/>
       </c>
       <c r="N3" t="str">
-        <v>2026-06-22</v>
+        <v>2026-06-20</v>
       </c>
       <c r="O3" t="str">
-        <v>2026-06-22</v>
+        <v>Pago</v>
       </c>
       <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
         <v>Sim</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Pago</v>
+        <v>D</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>26/06/2026 11:53:36</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D4" t="str">
-        <v>7xa6n9jf</v>
+        <v>lhli3ol0</v>
       </c>
       <c r="E4" t="str">
         <v>Despesa</v>
@@ -581,13 +590,13 @@
         <v>DPBEA</v>
       </c>
       <c r="I4" t="str">
-        <v>Diária: Sergio Tarnta — DPBEA (demolição)</v>
+        <v>Demolição</v>
       </c>
       <c r="J4">
         <v>200</v>
       </c>
       <c r="K4" t="str">
-        <v>PIX</v>
+        <v>À vista</v>
       </c>
       <c r="L4" t="str">
         <v/>
@@ -596,27 +605,30 @@
         <v/>
       </c>
       <c r="N4" t="str">
-        <v>2026-06-23</v>
+        <v>2026-06-22</v>
       </c>
       <c r="O4" t="str">
-        <v>2026-06-23</v>
+        <v>Pago</v>
       </c>
       <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
         <v>Sim</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Pago</v>
+        <v>D</v>
       </c>
       <c r="B5" t="str">
-        <v>24/06/2026 15:04:53</v>
+        <v>26/06/2026 11:53:38</v>
       </c>
       <c r="C5" t="str">
         <v>Administrador</v>
       </c>
       <c r="D5" t="str">
-        <v>5lahvabb</v>
+        <v>dqopqf8e</v>
       </c>
       <c r="E5" t="str">
         <v>Despesa</v>
@@ -628,47 +640,368 @@
         <v>Sergio Tarnta</v>
       </c>
       <c r="H5" t="str">
-        <v>Armazem - Cajamar</v>
+        <v>DPBEA</v>
       </c>
       <c r="I5" t="str">
-        <v>Diária: Sergio Tarnta — Armazem - Cajamar</v>
+        <v>Demolição</v>
       </c>
       <c r="J5">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="K5" t="str">
+        <v>À vista</v>
+      </c>
+      <c r="L5" t="str">
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>D</v>
+      </c>
+      <c r="B6" t="str">
+        <v>26/06/2026 11:53:40</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D6" t="str">
+        <v>4y0khrwr</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Despesa</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Mão de Obra</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Sergio Tarnta</v>
+      </c>
+      <c r="H6" t="str">
+        <v>DPBEA</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Demolição</v>
+      </c>
+      <c r="J6">
+        <v>200</v>
+      </c>
+      <c r="K6" t="str">
+        <v>À vista</v>
+      </c>
+      <c r="L6" t="str">
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-06-24</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>C</v>
+      </c>
+      <c r="B7" t="str">
+        <v>26/06/2026 12:08:24</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ra6tyffl</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Recebimento</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Notas Fiscais emitidas</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>DPBEA</v>
+      </c>
+      <c r="I7" t="str">
+        <v>Reforma</v>
+      </c>
+      <c r="J7">
+        <v>10000</v>
+      </c>
+      <c r="K7" t="str">
         <v>PIX</v>
       </c>
-      <c r="L5" t="str">
-        <v/>
-      </c>
-      <c r="M5" t="str">
-        <v/>
-      </c>
-      <c r="N5" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="O5" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="P5" t="str">
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
+      </c>
+      <c r="N7" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Recebido</v>
+      </c>
+      <c r="P7" t="str">
+        <v>2026-06-01</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>C</v>
+      </c>
+      <c r="B8" t="str">
+        <v>26/06/2026 12:08:56</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D8" t="str">
+        <v>yt4l7opi</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Recebimento</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Notas Fiscais emitidas</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Cajamar</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Instalação de divisória</v>
+      </c>
+      <c r="J8">
+        <v>20000</v>
+      </c>
+      <c r="K8" t="str">
+        <v>PIX</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
+      </c>
+      <c r="M8" t="str">
+        <v/>
+      </c>
+      <c r="N8" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Recebido</v>
+      </c>
+      <c r="P8" t="str">
+        <v>2026-06-02</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>C</v>
+      </c>
+      <c r="B9" t="str">
+        <v>26/06/2026 12:09:31</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D9" t="str">
+        <v>kt8qbtt9</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Despesa</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Mão de Obra</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Sergiio Tranta</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Cajamar</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Instalação de divisória</v>
+      </c>
+      <c r="J9">
+        <v>250</v>
+      </c>
+      <c r="K9" t="str">
+        <v>PIX</v>
+      </c>
+      <c r="L9" t="str">
+        <v/>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
+        <v>2026-06-20</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>C</v>
+      </c>
+      <c r="B10" t="str">
+        <v>26/06/2026 12:10:23</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D10" t="str">
+        <v>03tsvvto</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Despesa</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Mão de Obra</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Sergiio Tranta</v>
+      </c>
+      <c r="H10" t="str">
+        <v>DPBEA</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Demolição</v>
+      </c>
+      <c r="J10">
+        <v>200</v>
+      </c>
+      <c r="K10" t="str">
+        <v>PIX</v>
+      </c>
+      <c r="L10" t="str">
+        <v/>
+      </c>
+      <c r="M10" t="str">
+        <v/>
+      </c>
+      <c r="N10" t="str">
+        <v>2026-06-21</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="P10" t="str">
+        <v/>
+      </c>
+      <c r="Q10" t="str">
+        <v>Sim</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>C</v>
+      </c>
+      <c r="B11" t="str">
+        <v>26/06/2026 12:10:49</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D11" t="str">
+        <v>7yu7bkia</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Despesa</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Mão de Obra</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Sergiio Tranta</v>
+      </c>
+      <c r="H11" t="str">
+        <v>DPBEA</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Demolição</v>
+      </c>
+      <c r="J11">
+        <v>200</v>
+      </c>
+      <c r="K11" t="str">
+        <v>PIX</v>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
+      <c r="M11" t="str">
+        <v/>
+      </c>
+      <c r="N11" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Pago</v>
+      </c>
+      <c r="P11" t="str">
+        <v/>
+      </c>
+      <c r="Q11" t="str">
         <v>Sim</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Status</v>
+        <v>Status Auditoria</v>
       </c>
       <c r="B1" t="str">
         <v>Data/Hora</v>
@@ -697,13 +1030,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>D</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>26/06/2026 11:53:44</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D2" t="str">
         <v>Ob0001</v>
@@ -726,10 +1059,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>D</v>
       </c>
       <c r="B3" t="str">
-        <v>24/06/2026 14:43:00</v>
+        <v>26/06/2026 11:53:46</v>
       </c>
       <c r="C3" t="str">
         <v>Administrador</v>
@@ -753,16 +1086,74 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>C</v>
+      </c>
+      <c r="B4" t="str">
+        <v>26/06/2026 12:05:06</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Ob0003</v>
+      </c>
+      <c r="E4" t="str">
+        <v>DPBEA</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Reforma</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Nilce</v>
+      </c>
+      <c r="H4" t="str">
+        <v>19996494412</v>
+      </c>
+      <c r="I4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>C</v>
+      </c>
+      <c r="B5" t="str">
+        <v>26/06/2026 12:05:42</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Ob0004</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Cajamar</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Instalação de divisória</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Marcos Carvalho</v>
+      </c>
+      <c r="H5" t="str">
+        <v>19981749744</v>
+      </c>
+      <c r="I5">
+        <v>20000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -792,13 +1183,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>26/06/2026 11:53:50</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D2" t="str">
         <v>Col0001</v>
@@ -816,9 +1207,61 @@
         <v>Pintura, Marcenaria, Serralheria</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>D</v>
+      </c>
+      <c r="B3" t="str">
+        <v>26/06/2026 11:59:42</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Col0002</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Sergio Taranta</v>
+      </c>
+      <c r="F3" t="str">
+        <v>19999857226</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Campo Grande</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Pintura, Marcenaria, Serralheria</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>C</v>
+      </c>
+      <c r="B4" t="str">
+        <v>26/06/2026 12:06:22</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Administrador</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Col0003</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Sergiio Tranta</v>
+      </c>
+      <c r="F4" t="str">
+        <v>19999857226</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Campo Grande</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Pintura, Marcenaria, Serralheria</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -852,10 +1295,10 @@
         <v>C</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D2" t="str">
         <v>Cat0001</v>
@@ -872,10 +1315,10 @@
         <v>C</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D3" t="str">
         <v>Cat0002</v>
@@ -892,10 +1335,10 @@
         <v>C</v>
       </c>
       <c r="B4" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D4" t="str">
         <v>Cat0003</v>
@@ -912,10 +1355,10 @@
         <v>C</v>
       </c>
       <c r="B5" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D5" t="str">
         <v>Cat0004</v>
@@ -932,10 +1375,10 @@
         <v>C</v>
       </c>
       <c r="B6" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D6" t="str">
         <v>Cat0005</v>
@@ -952,10 +1395,10 @@
         <v>C</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D7" t="str">
         <v>Cat0006</v>
@@ -972,10 +1415,10 @@
         <v>C</v>
       </c>
       <c r="B8" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D8" t="str">
         <v>Cat0007</v>
@@ -992,10 +1435,10 @@
         <v>C</v>
       </c>
       <c r="B9" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D9" t="str">
         <v>Cat0008</v>
@@ -1012,10 +1455,10 @@
         <v>C</v>
       </c>
       <c r="B10" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D10" t="str">
         <v>Cat0009</v>
@@ -1032,10 +1475,10 @@
         <v>C</v>
       </c>
       <c r="B11" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D11" t="str">
         <v>Cat0010</v>
@@ -1052,10 +1495,10 @@
         <v>C</v>
       </c>
       <c r="B12" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D12" t="str">
         <v>Cat0011</v>
@@ -1072,10 +1515,10 @@
         <v>C</v>
       </c>
       <c r="B13" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D13" t="str">
         <v>Cat0012</v>
@@ -1092,10 +1535,10 @@
         <v>C</v>
       </c>
       <c r="B14" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D14" t="str">
         <v>Cat0013</v>
@@ -1112,10 +1555,10 @@
         <v>C</v>
       </c>
       <c r="B15" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D15" t="str">
         <v>Cat0014</v>
@@ -1132,10 +1575,10 @@
         <v>C</v>
       </c>
       <c r="B16" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C16" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D16" t="str">
         <v>Cat0015</v>
@@ -1152,10 +1595,10 @@
         <v>C</v>
       </c>
       <c r="B17" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C17" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D17" t="str">
         <v>Cat0016</v>
@@ -1172,10 +1615,10 @@
         <v>C</v>
       </c>
       <c r="B18" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C18" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D18" t="str">
         <v>Cat0017</v>
@@ -1192,10 +1635,10 @@
         <v>C</v>
       </c>
       <c r="B19" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C19" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D19" t="str">
         <v>Cat0018</v>
@@ -1212,10 +1655,10 @@
         <v>C</v>
       </c>
       <c r="B20" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C20" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D20" t="str">
         <v>Cat0019</v>
@@ -1232,10 +1675,10 @@
         <v>C</v>
       </c>
       <c r="B21" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C21" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D21" t="str">
         <v>Cat0020</v>
@@ -1252,10 +1695,10 @@
         <v>C</v>
       </c>
       <c r="B22" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C22" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D22" t="str">
         <v>Cat0021</v>
@@ -1272,10 +1715,10 @@
         <v>C</v>
       </c>
       <c r="B23" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C23" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D23" t="str">
         <v>Cat0022</v>
@@ -1292,10 +1735,10 @@
         <v>C</v>
       </c>
       <c r="B24" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C24" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D24" t="str">
         <v>Cat0023</v>
@@ -1312,10 +1755,10 @@
         <v>C</v>
       </c>
       <c r="B25" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C25" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D25" t="str">
         <v>Cat0024</v>
@@ -1332,10 +1775,10 @@
         <v>C</v>
       </c>
       <c r="B26" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C26" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D26" t="str">
         <v>Cat0025</v>
@@ -1352,10 +1795,10 @@
         <v>C</v>
       </c>
       <c r="B27" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C27" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D27" t="str">
         <v>Cat0026</v>
@@ -1372,10 +1815,10 @@
         <v>C</v>
       </c>
       <c r="B28" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C28" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D28" t="str">
         <v>Cat0027</v>
@@ -1392,10 +1835,10 @@
         <v>C</v>
       </c>
       <c r="B29" t="str">
-        <v/>
+        <v>—</v>
       </c>
       <c r="C29" t="str">
-        <v/>
+        <v>Sistema</v>
       </c>
       <c r="D29" t="str">
         <v>Cat0028</v>
@@ -1416,7 +1859,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1458,13 +1901,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="B2" t="str">
-        <v/>
+        <v>26/06/2026 12:01:14</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D2" t="str">
         <v>69ytk23o</v>
@@ -1496,13 +1939,13 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>C</v>
+        <v>D</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>26/06/2026 12:01:16</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Administrador</v>
       </c>
       <c r="D3" t="str">
         <v>xz4twdda</v>
@@ -1537,25 +1980,25 @@
         <v>D</v>
       </c>
       <c r="B4" t="str">
-        <v>24/06/2026 15:04:03</v>
+        <v>26/06/2026 12:01:18</v>
       </c>
       <c r="C4" t="str">
         <v>Administrador</v>
       </c>
       <c r="D4" t="str">
-        <v>bfx139lp</v>
+        <v>gziuoyj5</v>
       </c>
       <c r="E4" t="str">
         <v>Sergio Tarnta</v>
       </c>
       <c r="F4" t="str">
-        <v>DPBEA</v>
+        <v>Armazem - Cajamar</v>
       </c>
       <c r="G4" t="str">
         <v>2026-06-24</v>
       </c>
       <c r="H4">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="I4" t="str">
         <v>Pago</v>
@@ -1564,53 +2007,15 @@
         <v>PIX</v>
       </c>
       <c r="K4" t="str">
-        <v>demolição</v>
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>5mxjxyva</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>C</v>
-      </c>
-      <c r="B5" t="str">
-        <v>24/06/2026 15:04:53</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Administrador</v>
-      </c>
-      <c r="D5" t="str">
-        <v>gziuoyj5</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Sergio Tarnta</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Armazem - Cajamar</v>
-      </c>
-      <c r="G5" t="str">
-        <v>2026-06-24</v>
-      </c>
-      <c r="H5">
-        <v>300</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Pago</v>
-      </c>
-      <c r="J5" t="str">
-        <v>PIX</v>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
         <v>5lahvabb</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1667,7 +2072,7 @@
         <v>movimentacao</v>
       </c>
       <c r="B2" t="str">
-        <v>[{"tipo":"Recebimento","vencimento":"2026-06-24","catId":"Cat0013","valor":10000,"obraId":"Ob0001","colabId":null,"descricao":"NF 1234","formaPagamento":"À vista","pago":"Recebido","dataPag":"2026-06-20","parcelas":0,"numParcelas":null,"comprovante":null,"gerador":true,"id":"v2y7nnmu"},{"id":"dnspp1sf","tipo":"Despesa","catId":"Cat0015","colabId":"Col0001","obraId":"Ob0001","descricao":"Diária: Sergio Tarnta — DPBEA (Demolição)","valor":200,"formaPagamento":"PIX","pago":"Pago","dataPag":"2026-06-22","vencimento":"2026-06-22","parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"idParcelamento":null,"loop":0},{"id":"7xa6n9jf","tipo":"Despesa","catId":"Cat0015","colabId":"Col0001","obraId":"Ob0001","descricao":"Diária: Sergio Tarnta — DPBEA (demolição)","valor":200,"formaPagamento":"PIX","pago":"Pago","dataPag":"2026-06-23","vencimento":"2026-06-23","parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"idParcelamento":null,"loop":0},{"_status":"C","_auditAt":"24/06/2026 15:04:53","_auditUser":"Administrador","id":"5lahvabb","tipo":"Despesa","catId":"Cat0015","colabId":"Col0001","obraId":"Ob0002","descricao":"Diária: Sergio Tarnta — Armazem - Cajamar","valor":300,"formaPagamento":"PIX","pago":"Pago","dataPag":"2026-06-24","vencimento":"2026-06-24","parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"idParcelamento":null,"loop":0}]</v>
+        <v>[{"_status":"C","_auditAt":"26/06/2026 12:08:24","_auditUser":"Administrador","tipo":"Recebimento","vencimento":"2026-06-01","catId":"Cat0013","valor":10000,"obraId":"Ob0003","colabId":null,"descricao":"Reforma","formaPagamento":"PIX","pago":"Recebido","dataPag":"2026-06-01","parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"id":"ra6tyffl"},{"_status":"C","_auditAt":"26/06/2026 12:08:56","_auditUser":"Administrador","tipo":"Recebimento","vencimento":"2026-06-02","catId":"Cat0013","valor":20000,"obraId":"Ob0004","colabId":null,"descricao":"Instalação de divisória","formaPagamento":"PIX","pago":"Recebido","dataPag":"2026-06-02","parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"id":"yt4l7opi"},{"_status":"C","_auditAt":"26/06/2026 12:09:31","_auditUser":"Administrador","tipo":"Despesa","vencimento":"2026-06-20","catId":"Cat0015","valor":250,"obraId":"Ob0004","colabId":"Col0003","descricao":"Instalação de divisória","formaPagamento":"PIX","pago":"Pago","dataPag":null,"parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"id":"kt8qbtt9"},{"_status":"C","_auditAt":"26/06/2026 12:10:23","_auditUser":"Administrador","tipo":"Despesa","vencimento":"2026-06-21","catId":"Cat0015","valor":200,"obraId":"Ob0003","colabId":"Col0003","descricao":"Demolição","formaPagamento":"PIX","pago":"Pago","dataPag":null,"parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"id":"03tsvvto"},{"_status":"C","_auditAt":"26/06/2026 12:10:49","_auditUser":"Administrador","tipo":"Despesa","vencimento":"2026-06-23","catId":"Cat0015","valor":200,"obraId":"Ob0003","colabId":"Col0003","descricao":"Demolição","formaPagamento":"PIX","pago":"Pago","dataPag":null,"parcelas":0,"numParcelas":null,"comprovante":null,"compData":null,"gerador":true,"id":"7yu7bkia"}]</v>
       </c>
     </row>
     <row r="3">
@@ -1675,7 +2080,7 @@
         <v>obras</v>
       </c>
       <c r="B3" t="str">
-        <v>[{"nome":"DPBEA","contato":"Nilce","cel":"19996494412","descricao":"Departamento Público de Bem-Estar Animal","id":"Ob0001"},{"_status":"C","_auditAt":"24/06/2026 14:43:00","_auditUser":"Administrador","nome":"Armazem - Cajamar","contato":"Marcos Carvalho","cel":"19981749744","orcamento":null,"descricao":"Construção de divisória no arqmazem","id":"Ob0002"}]</v>
+        <v>[{"_status":"C","_auditAt":"26/06/2026 12:05:06","_auditUser":"Administrador","nome":"DPBEA","contato":"Nilce","cel":"19996494412","orcamento":10000,"descricao":"Reforma","id":"Ob0003"},{"_status":"C","_auditAt":"26/06/2026 12:05:42","_auditUser":"Administrador","nome":"Cajamar","contato":"Marcos Carvalho","cel":"19981749744","orcamento":20000,"descricao":"Instalação de divisória","id":"Ob0004"}]</v>
       </c>
     </row>
     <row r="4">
@@ -1683,7 +2088,7 @@
         <v>colaboradores</v>
       </c>
       <c r="B4" t="str">
-        <v>[{"nome":"Sergio Tarnta","contato":"19999857226","endereco":"Campo Grande","habilidades":"Pintura, Marcenaria, Serralheria","id":"Col0001"}]</v>
+        <v>[{"_status":"C","_auditAt":"26/06/2026 12:06:22","_auditUser":"Administrador","nome":"Sergiio Tranta","contato":"19999857226","endereco":"Campo Grande","habilidades":"Pintura, Marcenaria, Serralheria","id":"Col0003"}]</v>
       </c>
     </row>
     <row r="5">
@@ -1691,7 +2096,7 @@
         <v>categorias</v>
       </c>
       <c r="B5" t="str">
-        <v>[{"id":"Cat0001","nome":"Alimentação","tipo":"Despesa"},{"id":"Cat0002","nome":"Restaurantes","tipo":"Despesa"},{"id":"Cat0003","nome":"Compras","tipo":"Despesa"},{"id":"Cat0004","nome":"Mercado","tipo":"Despesa"},{"id":"Cat0005","nome":"Outros","tipo":"Despesa"},{"id":"Cat0006","nome":"Presentes e doações","tipo":"Despesa"},{"id":"Cat0007","nome":"Roupas","tipo":"Despesa"},{"id":"Cat0008","nome":"Saúde","tipo":"Despesa"},{"id":"Cat0009","nome":"Transporte","tipo":"Despesa"},{"id":"Cat0010","nome":"Viagem","tipo":"Despesa"},{"id":"Cat0011","nome":"Empréstimos","tipo":"Recebimento"},{"id":"Cat0012","nome":"Empresa","tipo":"Recebimento"},{"id":"Cat0013","nome":"Notas Fiscais emitidas","tipo":"Recebimento"},{"id":"Cat0014","nome":"Outras receitas","tipo":"Recebimento"},{"id":"Cat0015","nome":"Mão de Obra","tipo":"Despesa"},{"id":"Cat0016","nome":"Materiais de Construção","tipo":"Despesa"},{"id":"Cat0017","nome":"Equipamentos e Ferramentas","tipo":"Despesa"},{"id":"Cat0018","nome":"Subempreitada","tipo":"Despesa"},{"id":"Cat0019","nome":"Projetos e Consultoria","tipo":"Despesa"},{"id":"Cat0020","nome":"Transporte de Materiais","tipo":"Despesa"},{"id":"Cat0021","nome":"Licenças e Alvarás","tipo":"Despesa"},{"id":"Cat0022","nome":"Limpeza de Obra","tipo":"Despesa"},{"id":"Cat0023","nome":"Energia Elétrica (Obra)","tipo":"Despesa"},{"id":"Cat0024","nome":"Água (Obra)","tipo":"Despesa"},{"id":"Cat0025","nome":"EPI e Segurança","tipo":"Despesa"},{"id":"Cat0026","nome":"Despesas Administrativas","tipo":"Despesa"},{"id":"Cat0027","nome":"Receita de Obra","tipo":"Recebimento"},{"id":"Cat0028","nome":"Medição de Obra","tipo":"Recebimento"}]</v>
+        <v>[{"id":"Cat0001","nome":"Alimentação","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0002","nome":"Restaurantes","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0003","nome":"Compras","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0004","nome":"Mercado","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0005","nome":"Outros","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0006","nome":"Presentes e doações","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0007","nome":"Roupas","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0008","nome":"Saúde","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0009","nome":"Transporte","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0010","nome":"Viagem","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0011","nome":"Empréstimos","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0012","nome":"Empresa","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0013","nome":"Notas Fiscais emitidas","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0014","nome":"Outras receitas","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0015","nome":"Mão de Obra","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0016","nome":"Materiais de Construção","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0017","nome":"Equipamentos e Ferramentas","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0018","nome":"Subempreitada","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0019","nome":"Projetos e Consultoria","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0020","nome":"Transporte de Materiais","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0021","nome":"Licenças e Alvarás","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0022","nome":"Limpeza de Obra","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0023","nome":"Energia Elétrica (Obra)","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0024","nome":"Água (Obra)","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0025","nome":"EPI e Segurança","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0026","nome":"Despesas Administrativas","tipo":"Despesa","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0027","nome":"Receita de Obra","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"},{"id":"Cat0028","nome":"Medição de Obra","tipo":"Recebimento","_status":"C","_auditAt":"—","_auditUser":"Sistema"}]</v>
       </c>
     </row>
     <row r="6">
@@ -1699,7 +2104,7 @@
         <v>horas</v>
       </c>
       <c r="B6" t="str">
-        <v>[{"colabId":"Col0001","obraId":"Ob0001","data":"2026-06-22","diaria":200,"statusPag":"Pago","formaPagamento":"PIX","descricao":"Demolição","id":"69ytk23o","movId":"dnspp1sf"},{"colabId":"Col0001","obraId":"Ob0001","data":"2026-06-23","diaria":200,"statusPag":"Pago","formaPagamento":"PIX","descricao":"demolição","id":"xz4twdda","movId":"7xa6n9jf"},{"_status":"C","_auditAt":"24/06/2026 15:04:53","_auditUser":"Administrador","colabId":"Col0001","obraId":"Ob0002","data":"2026-06-24","diaria":300,"statusPag":"Pago","formaPagamento":"PIX","descricao":null,"id":"gziuoyj5","movId":"5lahvabb"}]</v>
+        <v>[]</v>
       </c>
     </row>
     <row r="7">
@@ -1731,7 +2136,7 @@
         <v>usuarios</v>
       </c>
       <c r="B10" t="str">
-        <v>[{"id":"u1","nome":"Administrador","usuario":"admin","senha":"1234","perfil":"admin"}]</v>
+        <v>[{"id":"u1","nome":"Administrador","usuario":"admin","perfil":"admin","salt":"hnfxplrxmuj50gwv","senhaHash":"97ed2d9e2011f2a3bf96a386e9a9456b69401ff1a2c7593c04c90382f424db49"}]</v>
       </c>
     </row>
   </sheetData>

</xml_diff>